<commit_message>
Split the Sprint 3 smoke run between the team as a relay
The Smoke run sheet gets a Who column (a dropdown that also takes free
text) assigning each step to the person playing that role, with the
coordinator's steps split between two people. Its note and the guide
describe running it as a relay on a call, each person logged in as
their own role(s). The Word copy of the guide is regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/regression/Sprint-3_Regression.xlsx
+++ b/docs/regression/Sprint-3_Regression.xlsx
@@ -924,11 +924,11 @@
         <v/>
       </c>
       <c r="C22" s="3">
-        <f>COUNTIF('Smoke run'!$F$5:$F$24,"Pass")</f>
+        <f>COUNTIF('Smoke run'!$G$5:$G$24,"Pass")</f>
         <v/>
       </c>
       <c r="D22" s="3">
-        <f>COUNTIF('Smoke run'!$F$5:$F$24,"Fail")</f>
+        <f>COUNTIF('Smoke run'!$G$5:$G$24,"Fail")</f>
         <v/>
       </c>
       <c r="E22" s="3" t="n"/>
@@ -1146,12 +1146,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1165,7 +1165,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Do this together on a call before splitting up. Take one new event, titled 'REG S3 &lt;your name&gt;', through the sprint goal end to end. Do not use any story's fixture events. Password for every account: password123. Use an event date about 4 weeks ahead, with times on the quarter hour (e.g. 10:00-12:00).</t>
+          <t>A relay on a call, before splitting up: each person stays logged in as their role(s) on their own laptop and does their steps when the event reaches them, in order. Take one new event, titled 'REG S3 Smoke', through the sprint goal end to end - do not use any story's fixture events. Password for every account: password123. Use an event date about 4 weeks ahead, with times on the quarter hour (e.g. 10:00-12:00). Change 'Who' if you swap roles.</t>
         </is>
       </c>
     </row>
@@ -1177,32 +1177,32 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
           <t>Role (log in as)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>What to do</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Stories</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Result</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>Tested by</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
@@ -1215,28 +1215,32 @@
       <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Kristen</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Event Organiser
 rachel.ng@meridianfina.com</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Create an event request with expected attendance 120. Save it as a draft, reopen it from My Events and submit it.</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Status is Submitted. My Events lists only Rachel's own events.</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>SPM-23, 24, 25, 31</t>
         </is>
       </c>
-      <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
     </row>
@@ -1244,28 +1248,32 @@
       <c r="A6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Kristen</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Event Operations Manager
 grace.lim@connectsphere.com</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Assignments: assign Daniel Tan to the event.</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Status is Under review. Rachel sees Daniel Tan as the coordinator.</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>SPM-30</t>
         </is>
       </c>
-      <c r="F6" s="4" t="n"/>
       <c r="G6" s="4" t="n"/>
       <c r="H6" s="4" t="n"/>
     </row>
@@ -1273,28 +1281,32 @@
       <c r="A7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Event Coordinator
 daniel.tan@connectsphere.com</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Review Queue: open the event, approve it, then begin planning.</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Status is Planning.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>SPM-28, 54</t>
         </is>
       </c>
-      <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n"/>
       <c r="H7" s="4" t="n"/>
     </row>
@@ -1302,27 +1314,31 @@
       <c r="A8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Event Coordinator</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Update the event information with an ordinary edit (e.g. the description only).</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>The change is saved. No arrangement is flagged and the status stays Planning.</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>SPM-62</t>
         </is>
       </c>
-      <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
     </row>
@@ -1330,27 +1346,31 @@
       <c r="A9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Event Coordinator</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Venue tab: request two venues for the same times: a main room (purpose "Main programme", 120 people) and a breakout room (purpose "Breakout", 40 people), each with its own layout.</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Both bookings show on the event as Pending, each with its own venue, purpose, times and hold expiry. Each venue was checked against its own attendance and layout.</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>SPM-40, 41, 42, 44, 81, 82, 90, 93</t>
         </is>
       </c>
-      <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="n"/>
     </row>
@@ -1358,27 +1378,31 @@
       <c r="A10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Event Coordinator</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Equipment tab: record one equipment requirement.</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>The requirement is saved and shows as Requested.</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>SPM-47</t>
         </is>
       </c>
-      <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="4" t="n"/>
     </row>
@@ -1386,28 +1410,32 @@
       <c r="A11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Kayalvizhi</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Technical Support Staff
 kenji.sato@connectsphere.com</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Equipment Requests: open the event's request, check availability and reserve it. Then mark one unrelated equipment item under maintenance and return it to available.</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>The request shows Reserved. The item's status changes and changes back.</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>SPM-48, 49, 50, 55</t>
         </is>
       </c>
-      <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="n"/>
     </row>
@@ -1415,28 +1443,32 @@
       <c r="A12" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Kayalvizhi</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Venue Staff
 marcus.wong@connectsphere.com</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Booking Requests: approve both of the event's requests.</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Each request shows its purpose, the requested times and the room in use including setup and turnaround. Both bookings are Approved.</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>SPM-43, 90, 93</t>
         </is>
       </c>
-      <c r="F12" s="4" t="n"/>
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="4" t="n"/>
     </row>
@@ -1444,27 +1476,31 @@
       <c r="A13" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Kayalvizhi</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Venue Staff</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Venues: mark the breakout room unavailable for a period that covers the event's times, with a reason.</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>The unavailable period shows on the venue's availability calendar.</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>SPM-45, 46</t>
         </is>
       </c>
-      <c r="F13" s="4" t="n"/>
       <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="n"/>
     </row>
@@ -1472,27 +1508,31 @@
       <c r="A14" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Event Coordinator</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Check Notifications, then open Flagged Arrangements.</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>The unread count is shown and a notification about the breakout room links to the event. Only the breakout booking is flagged, with the reason; the main room booking is unchanged.</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>SPM-45, 68, 71, 81</t>
         </is>
       </c>
-      <c r="F14" s="4" t="n"/>
       <c r="G14" s="4" t="n"/>
       <c r="H14" s="4" t="n"/>
     </row>
@@ -1500,27 +1540,31 @@
       <c r="A15" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Event Coordinator</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>From the flagged booking, search for a replacement venue, request it, then release the flagged booking with a reason.</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>The search is pre-filled from the flagged booking. The old booking shows Released and stays on the event. The event's own information and status do not change.</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>SPM-67, 68</t>
         </is>
       </c>
-      <c r="F15" s="4" t="n"/>
       <c r="G15" s="4" t="n"/>
       <c r="H15" s="4" t="n"/>
     </row>
@@ -1528,27 +1572,31 @@
       <c r="A16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Kayalvizhi</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Venue Staff</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Approve the replacement booking request.</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>The replacement booking is Approved. The released booking's time is free on its venue's calendar.</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>SPM-43, 67</t>
         </is>
       </c>
-      <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
       <c r="H16" s="4" t="n"/>
     </row>
@@ -1556,27 +1604,31 @@
       <c r="A17" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Event Coordinator</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>Turn on registration: capacity 100, measured against the main room booking, opening today and closing before the event. Then open Readiness and try to confirm the event.</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Readiness lists each venue booking separately, and the equipment, as done. Confirmation is refused and the Operational Safety Check is named as outstanding.</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>SPM-33, 34, 64, 88</t>
         </is>
       </c>
-      <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
       <c r="H17" s="4" t="n"/>
     </row>
@@ -1584,27 +1636,31 @@
       <c r="A18" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Event Coordinator</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>Submit the event for a safety check.</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Status is Safety review, and Rachel sees it as well.</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>SPM-86</t>
         </is>
       </c>
-      <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
       <c r="H18" s="4" t="n"/>
     </row>
@@ -1612,28 +1668,32 @@
       <c r="A19" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Safety Officer
 hana.yusof@connectsphere.com</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>Safety Checks: open the event and request changes, describing what is needed.</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>The sidebar shows only Dashboard, Safety Checks, All Events and Notifications. The review shows attendance, each venue with capacity and layout, and the equipment. Status returns to Planning.</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>SPM-85, 87</t>
         </is>
       </c>
-      <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
       <c r="H19" s="4" t="n"/>
     </row>
@@ -1641,27 +1701,31 @@
       <c r="A20" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Sammi, then Kristen</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Event Coordinator, then Event Organiser</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>Coordinator: read the decision on the event, then submit it for a safety check again. Organiser: open the event.</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>The coordinator sees the changes required. The organiser does not see the Safety Officer's reason. Status is Safety review again.</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>SPM-86, 88</t>
         </is>
       </c>
-      <c r="F20" s="4" t="n"/>
       <c r="G20" s="4" t="n"/>
       <c r="H20" s="4" t="n"/>
     </row>
@@ -1669,27 +1733,31 @@
       <c r="A21" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Janelle, then Sammi</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Safety Officer, then Event Coordinator</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>Safety Officer: approve the event. Coordinator: confirm the event.</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Status is Safety approved, then Confirmed.</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>SPM-34, 87, 88</t>
         </is>
       </c>
-      <c r="F21" s="4" t="n"/>
       <c r="G21" s="4" t="n"/>
       <c r="H21" s="4" t="n"/>
     </row>
@@ -1697,28 +1765,32 @@
       <c r="A22" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Attendee
 lee.wei.ming@example.com</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>Browse Events: find the event and register. Open My Registrations. Then withdraw the registration.</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>The registration shows Registered, then Withdrawn. The place is given back.</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>SPM-51, 52</t>
         </is>
       </c>
-      <c r="F22" s="4" t="n"/>
       <c r="G22" s="4" t="n"/>
       <c r="H22" s="4" t="n"/>
     </row>
@@ -1726,27 +1798,31 @@
       <c r="A23" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Kristen and Sammi</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Event Organiser and Event Coordinator</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>Each opens the event's Attendees tab.</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Lee Wei Ming is listed as Withdrawn, with the active count against the capacity of 100. Venue Staff and Technical Support have no Attendees tab.</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>SPM-65</t>
         </is>
       </c>
-      <c r="F23" s="4" t="n"/>
       <c r="G23" s="4" t="n"/>
       <c r="H23" s="4" t="n"/>
     </row>
@@ -1754,32 +1830,36 @@
       <c r="A24" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Everyone</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Every role</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>Log in as each role in turn.</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Each role sees only its own sidebar links (organiser "My Events"; coordinator, Ops Manager and Safety Officer "All Events"), and the organiser sees only their own events.</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>SPM-21, 22</t>
         </is>
       </c>
-      <c r="F24" s="4" t="n"/>
       <c r="G24" s="4" t="n"/>
       <c r="H24" s="4" t="n"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F5:F24">
+  <conditionalFormatting sqref="G5:G24">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1787,9 +1867,12 @@
       <formula>"Fail"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation sqref="F5:F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="G5:G24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B5:B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Kayalvizhi,Jordan,Janelle,Sammi,Kristen,Everyone"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix SPM-47 steps and warn against reseeding in the Sprint 3 tracker
SPM-47's test cases store their steps as one numbered string, which the
builder numbered character by character ("1. 1", "2. ."). They now
appear as written. Nine SPM-47/48/49 cases, written before the fixture
scripts existed, say their data comes from npx prisma db seed or to
reseed between cases; their rows now start with a warning not to, and
to mark the case Blocked if the data no longer matches.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/regression/Sprint-3_Regression.xlsx
+++ b/docs/regression/Sprint-3_Regression.xlsx
@@ -10461,270 +10461,12 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>1. 1
-2. .
-3.  
-4. O
-5. p
-6. e
-7. n
-8.  
-9. '
-10. P
-11. e
-12. a
-13. r
-14. l
-15.  
-16. D
-17. e
-18. l
-19. t
-20. a
-21.  
-22. S
-23. a
-24. f
-25. e
-26. t
-27. y
-28.  
-29. C
-30. o
-31. n
-32. f
-33. e
-34. r
-35. e
-36. n
-37. c
-38. e
-39. '
-40. 
-41. 2
-42. .
-43.  
-44. C
-45. l
-46. i
-47. c
-48. k
-49.  
-50. t
-51. h
-52. e
-53.  
-54. '
-55. E
-56. q
-57. u
-58. i
-59. p
-60. m
-61. e
-62. n
-63. t
-64. '
-65.  
-66. t
-67. a
-68. b
-69. 
-70. 3
-71. .
-72.  
-73. I
-74. n
-75.  
-76. '
-77. A
-78. d
-79. d
-80.  
-81. e
-82. q
-83. u
-84. i
-85. p
-86. m
-87. e
-88. n
-89. t
-90. '
-91. ,
-92.  
-93. o
-94. p
-95. e
-96. n
-97.  
-98. t
-99. h
-100. e
-101.  
-102. '
-103. E
-104. q
-105. u
-106. i
-107. p
-108. m
-109. e
-110. n
-111. t
-112. '
-113.  
-114. d
-115. r
-116. o
-117. p
-118. d
-119. o
-120. w
-121. n
-122.  
-123. a
-124. n
-125. d
-126.  
-127. c
-128. h
-129. o
-130. o
-131. s
-132. e
-133.  
-134. '
-135. H
-136. a
-137. n
-138. d
-139. h
-140. e
-141. l
-142. d
-143.  
-144. W
-145. i
-146. r
-147. e
-148. l
-149. e
-150. s
-151. s
-152.  
-153. M
-154. i
-155. c
-156. '
-157. 
-158. 4
-159. .
-160.  
-161. S
-162. e
-163. t
-164.  
-165. '
-166. Q
-167. u
-168. a
-169. n
-170. t
-171. i
-172. t
-173. y
-174. '
-175.  
-176. t
-177. o
-178.  
-179. 6
-180. 
-181. 5
-182. .
-183.  
-184. E
-185. n
-186. t
-187. e
-188. r
-189.  
-190. '
-191. L
-192. a
-193. p
-194. e
-195. l
-196.  
-197. m
-198. i
-199. c
-200. s
-201.  
-202. f
-203. o
-204. r
-205.  
-206. p
-207. a
-208. n
-209. e
-210. l
-211.  
-212. s
-213. p
-214. e
-215. a
-216. k
-217. e
-218. r
-219. s
-220. .
-221. '
-222.  
-223. i
-224. n
-225.  
-226. '
-227. T
-228. e
-229. c
-230. h
-231. n
-232. i
-233. c
-234. a
-235. l
-236.  
-237. r
-238. e
-239. q
-240. u
-241. i
-242. r
-243. e
-244. m
-245. e
-246. n
-247. t
-248. s
-249. '
-250. 
-251. 6
-252. .
-253.  
-254. C
-255. l
-256. i
-257. c
-258. k
-259.  
-260. '
-261. A
-262. d
-263. d
-264. '</t>
+          <t>1. Open 'Pearl Delta Safety Conference'
+2. Click the 'Equipment' tab
+3. In 'Add equipment', open the 'Equipment' dropdown and choose 'Handheld Wireless Mic'
+4. Set 'Quantity' to 6
+5. Enter 'Lapel mics for panel speakers.' in 'Technical requirements'
+6. Click 'Add'</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -10776,91 +10518,8 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>1. 1
-2. .
-3.  
-4. O
-5. p
-6. e
-7. n
-8.  
-9. '
-10. P
-11. e
-12. a
-13. r
-14. l
-15.  
-16. D
-17. e
-18. l
-19. t
-20. a
-21.  
-22. S
-23. a
-24. f
-25. e
-26. t
-27. y
-28.  
-29. C
-30. o
-31. n
-32. f
-33. e
-34. r
-35. e
-36. n
-37. c
-38. e
-39. '
-40.  
-41. f
-42. r
-43. o
-44. m
-45.  
-46. '
-47. M
-48. y
-49.  
-50. E
-51. v
-52. e
-53. n
-54. t
-55. s
-56. '
-57. 
-58. 2
-59. .
-60.  
-61. C
-62. l
-63. i
-64. c
-65. k
-66.  
-67. t
-68. h
-69. e
-70.  
-71. '
-72. E
-73. q
-74. u
-75. i
-76. p
-77. m
-78. e
-79. n
-80. t
-81. '
-82.  
-83. t
-84. a
-85. b</t>
+          <t>1. Open 'Pearl Delta Safety Conference' from 'My Events'
+2. Click the 'Equipment' tab</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
@@ -10899,7 +10558,8 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Logged in as Hui Shan Neo (huishan.neo@connectsphere.com / password123), Coordinator of 'Pearl Delta Safety Conference'.
+          <t>DO NOT run npx prisma db seed, whatever the text below says - it wipes the shared database. Use the base seed data as it is; if it no longer matches, mark the case Blocked.
+Logged in as Hui Shan Neo (huishan.neo@connectsphere.com / password123), Coordinator of 'Pearl Delta Safety Conference'.
 The event has two sessions: 'Morning briefing' (09:00-12:00) and 'Afternoon workshop' (13:00-17:00), both on 14 Dec 2026. There is no in-app way to add a session to an existing event, so both sessions are seeded by `npx prisma db seed`.</t>
         </is>
       </c>
@@ -10910,323 +10570,11 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>1. 1
-2. .
-3.  
-4. O
-5. p
-6. e
-7. n
-8.  
-9. t
-10. h
-11. e
-12.  
-13. '
-14. E
-15. q
-16. u
-17. i
-18. p
-19. m
-20. e
-21. n
-22. t
-23. '
-24.  
-25. t
-26. a
-27. b
-28.  
-29. o
-30. f
-31.  
-32. '
-33. P
-34. e
-35. a
-36. r
-37. l
-38.  
-39. D
-40. e
-41. l
-42. t
-43. a
-44.  
-45. S
-46. a
-47. f
-48. e
-49. t
-50. y
-51.  
-52. C
-53. o
-54. n
-55. f
-56. e
-57. r
-58. e
-59. n
-60. c
-61. e
-62. '
-63. 
-64. 2
-65. .
-66.  
-67. I
-68. n
-69.  
-70. '
-71. A
-72. d
-73. d
-74.  
-75. e
-76. q
-77. u
-78. i
-79. p
-80. m
-81. e
-82. n
-83. t
-84. '
-85. ,
-86.  
-87. c
-88. h
-89. o
-90. o
-91. s
-92. e
-93.  
-94. '
-95. G
-96. o
-97. o
-98. s
-99. e
-100. n
-101. e
-102. c
-103. k
-104.  
-105. T
-106. a
-107. b
-108. l
-109. e
-110.  
-111. M
-112. i
-113. c
-114. '
-115. ,
-116.  
-117. s
-118. e
-119. t
-120.  
-121. Q
-122. u
-123. a
-124. n
-125. t
-126. i
-127. t
-128. y
-129.  
-130. t
-131. o
-132.  
-133. 1
-134. ,
-135.  
-136. a
-137. n
-138. d
-139.  
-140. c
-141. h
-142. o
-143. o
-144. s
-145. e
-146.  
-147. '
-148. M
-149. o
-150. r
-151. n
-152. i
-153. n
-154. g
-155.  
-156. b
-157. r
-158. i
-159. e
-160. f
-161. i
-162. n
-163. g
-164. '
-165.  
-166. i
-167. n
-168.  
-169. t
-170. h
-171. e
-172.  
-173. n
-174. e
-175. w
-176.  
-177. '
-178. S
-179. e
-180. s
-181. s
-182. i
-183. o
-184. n
-185. '
-186.  
-187. d
-188. r
-189. o
-190. p
-191. d
-192. o
-193. w
-194. n
-195. 
-196. 3
-197. .
-198.  
-199. C
-200. l
-201. i
-202. c
-203. k
-204.  
-205. '
-206. A
-207. d
-208. d
-209. '
-210. 
-211. 4
-212. .
-213.  
-214. C
-215. h
-216. o
-217. o
-218. s
-219. e
-220.  
-221. '
-222. P
-223. o
-224. w
-225. e
-226. r
-227. e
-228. d
-229.  
-230. S
-231. p
-232. e
-233. a
-234. k
-235. e
-236. r
-237. '
-238. ,
-239.  
-240. s
-241. e
-242. t
-243.  
-244. Q
-245. u
-246. a
-247. n
-248. t
-249. i
-250. t
-251. y
-252.  
-253. t
-254. o
-255.  
-256. 2
-257. ,
-258.  
-259. a
-260. n
-261. d
-262.  
-263. c
-264. h
-265. o
-266. o
-267. s
-268. e
-269.  
-270. '
-271. A
-272. f
-273. t
-274. e
-275. r
-276. n
-277. o
-278. o
-279. n
-280.  
-281. w
-282. o
-283. r
-284. k
-285. s
-286. h
-287. o
-288. p
-289. '
-290.  
-291. i
-292. n
-293.  
-294. '
-295. S
-296. e
-297. s
-298. s
-299. i
-300. o
-301. n
-302. '
-303. 
-304. 5
-305. .
-306.  
-307. C
-308. l
-309. i
-310. c
-311. k
-312.  
-313. '
-314. A
-315. d
-316. d
-317. '</t>
+          <t>1. Open the 'Equipment' tab of 'Pearl Delta Safety Conference'
+2. In 'Add equipment', choose 'Gooseneck Table Mic', set Quantity to 1, and choose 'Morning briefing' in the new 'Session' dropdown
+3. Click 'Add'
+4. Choose 'Powered Speaker', set Quantity to 2, and choose 'Afternoon workshop' in 'Session'
+5. Click 'Add'</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -11283,7 +10631,8 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>'Stage Wash Light': 2 total, 0 in maintenance.
+          <t>DO NOT run npx prisma db seed, whatever the text below says - it wipes the shared database. Use the base seed data as it is; if it no longer matches, mark the case Blocked.
+'Stage Wash Light': 2 total, 0 in maintenance.
 Event 'Morning Workshop' (2026-12-01, 09:00-12:00) holds 1x Stage Wash Light.
 Event 'Evening Recital' (2026-12-01, 18:00-21:00) requests 1x Stage Wash Light.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
@@ -11338,7 +10687,8 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Rule source: customer Q&amp;A #74 (different sessions can have different equipment) and SPM-47.
+          <t>DO NOT run npx prisma db seed, whatever the text below says - it wipes the shared database. Use the base seed data as it is; if it no longer matches, mark the case Blocked.
+Rule source: customer Q&amp;A #74 (different sessions can have different equipment) and SPM-47.
 'PA Speaker': 2 total, 0 in maintenance.
 Event 'Open House' (2026-10-05) holds 2x PA Speaker.
 Event 'Two-Day Summit' has session 'Day 1' (2026-10-05) and session 'Day 2' (2026-10-20). Each session requests 2x PA Speaker.
@@ -11451,7 +10801,8 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>'Document Camera': 5 total with 2 recorded as in maintenance, none reserved elsewhere.
+          <t>DO NOT run npx prisma db seed, whatever the text below says - it wipes the shared database. Use the base seed data as it is; if it no longer matches, mark the case Blocked.
+'Document Camera': 5 total with 2 recorded as in maintenance, none reserved elsewhere.
 Event 'Alumni Talk' (2026-10-28) requests 3x Document Camera.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).
@@ -11506,7 +10857,8 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Event 'Vendor Networking Evening' (2026-11-15, 17:00-22:00, booked at Marina Grand Hall) requests 6x Lavalier Wireless Mic, 1x Streaming Encoder, 2x Truss Lighting Bar and 1x Marina Hall Sound System.
+          <t>DO NOT run npx prisma db seed, whatever the text below says - it wipes the shared database. Use the base seed data as it is; if it no longer matches, mark the case Blocked.
+Event 'Vendor Networking Evening' (2026-11-15, 17:00-22:00, booked at Marina Grand Hall) requests 6x Lavalier Wireless Mic, 1x Streaming Encoder, 2x Truss Lighting Bar and 1x Marina Hall Sound System.
 Stock for those dates: Lavalier Wireless Mic 10 total, 2 in maintenance, 4 held by 'Regional Tech Expo' (2026-11-14). Streaming Encoder 3 total, 2 held by 'Regional Tech Expo' and 1 by 'Annual Partner Awards Night' (2026-11-16). Truss Lighting Bar 6 total, 1 in maintenance. Marina Hall Sound System 1 total, kept at Marina Grand Hall.
 Data: seeded by `npx prisma db seed` (SPM-48 test fixtures).
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
@@ -11582,7 +10934,8 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Rule (team decision): clicking Reserve always reserves the smaller of what was requested and what is available for that line - never more than requested, and never more than available. There is no quantity box to type into.
+          <t>DO NOT run npx prisma db seed, whatever the text below says - it wipes the shared database. Use the base seed data as it is; if it no longer matches, mark the case Blocked.
+Rule (team decision): clicking Reserve always reserves the smaller of what was requested and what is available for that line - never more than requested, and never more than available. There is no quantity box to type into.
 'Portable Stage': 6 total, 0 in maintenance, none held by other events for these dates.
 Event 'Spring Fair' (2027-02-02) requests 3x Portable Stage (status 'Under review').
 Data: seeded by `npx prisma db seed` (SPM-49 test fixtures). Every case that reserves changes the data, so reseed before running it again.
@@ -11639,7 +10992,8 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>'Portable Stage': 6 total, 0 in maintenance, none held by other events for these dates.
+          <t>DO NOT run npx prisma db seed, whatever the text below says - it wipes the shared database. Use the base seed data as it is; if it no longer matches, mark the case Blocked.
+'Portable Stage': 6 total, 0 in maintenance, none held by other events for these dates.
 Event 'Autumn Fair' (2027-02-09) requests 2x Portable Stage.
 Data: seeded by `npx prisma db seed` (SPM-49 test fixtures). Every case that reserves changes the data, so reseed before running it again.
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
@@ -11695,7 +11049,8 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Rule source: customer Q&amp;A #74 (sessions can need different equipment).
+          <t>DO NOT run npx prisma db seed, whatever the text below says - it wipes the shared database. Use the base seed data as it is; if it no longer matches, mark the case Blocked.
+Rule source: customer Q&amp;A #74 (sessions can need different equipment).
 'Wireless Presenter': 4 total, 0 in maintenance. Event 'Trade Mixer' (2027-06-07) already holds all 4 (reserved).
 Event 'Two-Day Forum' has session 'Day 1' (2027-06-07) and session 'Day 2' (2027-06-21), each requesting 2x Wireless Presenter.
 Data: seeded by `npx prisma db seed` (SPM-49 test fixtures). Every case that reserves changes the data, so reseed before running it again.
@@ -11754,7 +11109,8 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>Rule source: customer Q&amp;A #66 (Technical Support is not restricted by equipment type or location).
+          <t>DO NOT run npx prisma db seed, whatever the text below says - it wipes the shared database. Use the base seed data as it is; if it no longer matches, mark the case Blocked.
+Rule source: customer Q&amp;A #66 (Technical Support is not restricted by equipment type or location).
 'Portable Stage': 6 total, 0 in maintenance.
 Event 'Reserved Showcase' (2027-07-05) already has a reservation for 3x Portable Stage (status 'Reserved'), made by another Technical Support user.
 Data: seeded by `npx prisma db seed` (SPM-49 test fixtures).

</xml_diff>